<commit_message>
Update data: 3 Agustus 2026 pukul 12.40 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2 Juli" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Juli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 10 Agustus 2026 pukul 08.13 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data mikro SLS, report generator, and dashboard sync
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 11 Agustus 2026 pukul 07.41 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="10 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 12 Agustus 2026 pukul 06.53 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="11 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 13 Agustus 2026 pukul 07.47 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="12 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 14 Agustus 2026 pukul 07.06 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="13 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>

<commit_message>
Update data: 17 Agustus 2026 pukul 07.46 WITA
</commit_message>
<xml_diff>
--- a/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
+++ b/dashboard/public/Monev_Pendataan_SE2026_Morning.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="16 Agustus" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Agustus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PPL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progres PML" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Muatan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kecamatan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rekap Kecamatan" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progres PPL'!$A$3:$AO$3</definedName>

</xml_diff>